<commit_message>
Replace manual changelog notes with auto git_commits column
Rename picks.xlsx 'notes' column to 'git_commits' (last column). Replace
the manual log_model_change/changelog.json mechanism — which was never
auto-populated — with _get_git_commits_for_model(), which queries git log
over the 14 days before each pick date and filters commits by model-specific
keywords so each row reflects actual code changes.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/picks.xlsx
+++ b/tracking/picks.xlsx
@@ -497,12 +497,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>pnl_50</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>pnl_50</t>
+          <t>git_commits</t>
         </is>
       </c>
     </row>
@@ -532,7 +532,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>100</v>
       </c>
@@ -555,8 +554,7 @@
       <c r="L2" t="n">
         <v>-100</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
+      <c r="M2" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -609,8 +607,7 @@
       <c r="L3" t="n">
         <v>-100</v>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="n">
+      <c r="M3" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -663,8 +660,7 @@
       <c r="L4" t="n">
         <v>62.7</v>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
+      <c r="M4" t="n">
         <v>31.35</v>
       </c>
     </row>
@@ -717,8 +713,7 @@
       <c r="L5" t="n">
         <v>95.23999999999999</v>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="n">
+      <c r="M5" t="n">
         <v>47.62</v>
       </c>
     </row>
@@ -771,8 +766,7 @@
       <c r="L6" t="n">
         <v>-100</v>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="n">
+      <c r="M6" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -825,8 +819,7 @@
       <c r="L7" t="n">
         <v>60.61</v>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
+      <c r="M7" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -879,8 +872,7 @@
       <c r="L8" t="n">
         <v>86.95999999999999</v>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="n">
+      <c r="M8" t="n">
         <v>43.48</v>
       </c>
     </row>
@@ -933,8 +925,7 @@
       <c r="L9" t="n">
         <v>-100</v>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="n">
+      <c r="M9" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -987,8 +978,7 @@
       <c r="L10" t="n">
         <v>100</v>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="n">
+      <c r="M10" t="n">
         <v>50</v>
       </c>
     </row>
@@ -1018,7 +1008,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>-157.5</v>
       </c>
@@ -1041,8 +1030,7 @@
       <c r="L11" t="n">
         <v>63.49</v>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="n">
+      <c r="M11" t="n">
         <v>31.75</v>
       </c>
     </row>
@@ -1089,10 +1077,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1143,8 +1127,7 @@
       <c r="L13" t="n">
         <v>62.11</v>
       </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="n">
+      <c r="M13" t="n">
         <v>31.06</v>
       </c>
     </row>
@@ -1191,10 +1174,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1222,7 +1201,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
         <v>120</v>
       </c>
@@ -1245,8 +1223,7 @@
       <c r="L15" t="n">
         <v>-100</v>
       </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="n">
+      <c r="M15" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -1276,7 +1253,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
         <v>-141.5</v>
       </c>
@@ -1299,8 +1275,7 @@
       <c r="L16" t="n">
         <v>70.67</v>
       </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
+      <c r="M16" t="n">
         <v>35.34</v>
       </c>
     </row>
@@ -1330,7 +1305,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
         <v>-121</v>
       </c>
@@ -1353,8 +1327,7 @@
       <c r="L17" t="n">
         <v>82.64</v>
       </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="n">
+      <c r="M17" t="n">
         <v>41.32</v>
       </c>
     </row>
@@ -1407,8 +1380,7 @@
       <c r="L18" t="n">
         <v>95.23999999999999</v>
       </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="n">
+      <c r="M18" t="n">
         <v>47.62</v>
       </c>
     </row>
@@ -1461,8 +1433,7 @@
       <c r="L19" t="n">
         <v>82.64</v>
       </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="n">
+      <c r="M19" t="n">
         <v>41.32</v>
       </c>
     </row>
@@ -1515,8 +1486,7 @@
       <c r="L20" t="n">
         <v>94.34</v>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="n">
+      <c r="M20" t="n">
         <v>47.17</v>
       </c>
     </row>
@@ -1569,8 +1539,7 @@
       <c r="L21" t="n">
         <v>86.95999999999999</v>
       </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
+      <c r="M21" t="n">
         <v>43.48</v>
       </c>
     </row>
@@ -1617,10 +1586,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1671,8 +1636,7 @@
       <c r="L23" t="n">
         <v>-100</v>
       </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="n">
+      <c r="M23" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -1725,8 +1689,7 @@
       <c r="L24" t="n">
         <v>-100</v>
       </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="n">
+      <c r="M24" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -1779,8 +1742,7 @@
       <c r="L25" t="n">
         <v>70.92</v>
       </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="n">
+      <c r="M25" t="n">
         <v>35.46</v>
       </c>
     </row>
@@ -1833,8 +1795,7 @@
       <c r="L26" t="n">
         <v>-100</v>
       </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="n">
+      <c r="M26" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -1887,8 +1848,7 @@
       <c r="L27" t="n">
         <v>-100</v>
       </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="n">
+      <c r="M27" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -1941,8 +1901,7 @@
       <c r="L28" t="n">
         <v>65.15000000000001</v>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="n">
+      <c r="M28" t="n">
         <v>32.57</v>
       </c>
     </row>
@@ -1995,8 +1954,7 @@
       <c r="L29" t="n">
         <v>-100</v>
       </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="n">
+      <c r="M29" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -2049,8 +2007,7 @@
       <c r="L30" t="n">
         <v>66.67</v>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="n">
+      <c r="M30" t="n">
         <v>33.33</v>
       </c>
     </row>
@@ -2103,8 +2060,7 @@
       <c r="L31" t="n">
         <v>57.14</v>
       </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="n">
+      <c r="M31" t="n">
         <v>28.57</v>
       </c>
     </row>
@@ -2157,8 +2113,7 @@
       <c r="L32" t="n">
         <v>73.8</v>
       </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="n">
+      <c r="M32" t="n">
         <v>36.9</v>
       </c>
     </row>
@@ -2211,8 +2166,7 @@
       <c r="L33" t="n">
         <v>-100</v>
       </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="n">
+      <c r="M33" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -2265,8 +2219,7 @@
       <c r="L34" t="n">
         <v>-100</v>
       </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="n">
+      <c r="M34" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -2319,8 +2272,7 @@
       <c r="L35" t="n">
         <v>-100</v>
       </c>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="n">
+      <c r="M35" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -2373,8 +2325,7 @@
       <c r="L36" t="n">
         <v>-100</v>
       </c>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="n">
+      <c r="M36" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -2427,8 +2378,7 @@
       <c r="L37" t="n">
         <v>-100</v>
       </c>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="n">
+      <c r="M37" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -2481,8 +2431,7 @@
       <c r="L38" t="n">
         <v>54.05</v>
       </c>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="n">
+      <c r="M38" t="n">
         <v>27.03</v>
       </c>
     </row>
@@ -2535,8 +2484,7 @@
       <c r="L39" t="n">
         <v>80</v>
       </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="n">
+      <c r="M39" t="n">
         <v>40</v>
       </c>
     </row>
@@ -2589,8 +2537,7 @@
       <c r="L40" t="n">
         <v>-100</v>
       </c>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="n">
+      <c r="M40" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -2643,8 +2590,7 @@
       <c r="L41" t="n">
         <v>58.82</v>
       </c>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="n">
+      <c r="M41" t="n">
         <v>29.41</v>
       </c>
     </row>
@@ -2697,8 +2643,7 @@
       <c r="L42" t="n">
         <v>57.14</v>
       </c>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="n">
+      <c r="M42" t="n">
         <v>28.57</v>
       </c>
     </row>
@@ -2751,8 +2696,7 @@
       <c r="L43" t="n">
         <v>145</v>
       </c>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="n">
+      <c r="M43" t="n">
         <v>72.5</v>
       </c>
     </row>
@@ -2805,8 +2749,7 @@
       <c r="L44" t="n">
         <v>-100</v>
       </c>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="n">
+      <c r="M44" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -2859,8 +2802,7 @@
       <c r="L45" t="n">
         <v>90.91</v>
       </c>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="n">
+      <c r="M45" t="n">
         <v>45.45</v>
       </c>
     </row>
@@ -2913,8 +2855,7 @@
       <c r="L46" t="n">
         <v>-100</v>
       </c>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="n">
+      <c r="M46" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -2961,10 +2902,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr"/>
-      <c r="L47" t="inlineStr"/>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3015,8 +2952,7 @@
       <c r="L48" t="n">
         <v>59.7</v>
       </c>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="n">
+      <c r="M48" t="n">
         <v>29.85</v>
       </c>
     </row>
@@ -3069,8 +3005,7 @@
       <c r="L49" t="n">
         <v>-100</v>
       </c>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="n">
+      <c r="M49" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -3123,8 +3058,7 @@
       <c r="L50" t="n">
         <v>-100</v>
       </c>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="n">
+      <c r="M50" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -3154,7 +3088,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr"/>
       <c r="G51" t="n">
         <v>120</v>
       </c>
@@ -3177,8 +3110,7 @@
       <c r="L51" t="n">
         <v>120</v>
       </c>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="n">
+      <c r="M51" t="n">
         <v>60</v>
       </c>
     </row>
@@ -3208,7 +3140,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr"/>
       <c r="G52" t="n">
         <v>-102</v>
       </c>
@@ -3231,8 +3162,7 @@
       <c r="L52" t="n">
         <v>98.04000000000001</v>
       </c>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="n">
+      <c r="M52" t="n">
         <v>49.02</v>
       </c>
     </row>
@@ -3262,7 +3192,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr"/>
       <c r="G53" t="n">
         <v>-112</v>
       </c>
@@ -3285,8 +3214,7 @@
       <c r="L53" t="n">
         <v>-100</v>
       </c>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="n">
+      <c r="M53" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -3316,7 +3244,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr"/>
       <c r="G54" t="n">
         <v>106</v>
       </c>
@@ -3339,8 +3266,7 @@
       <c r="L54" t="n">
         <v>-100</v>
       </c>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="n">
+      <c r="M54" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -3370,7 +3296,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="n">
         <v>-156.5</v>
       </c>
@@ -3393,8 +3318,7 @@
       <c r="L55" t="n">
         <v>63.9</v>
       </c>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="n">
+      <c r="M55" t="n">
         <v>31.95</v>
       </c>
     </row>
@@ -3424,7 +3348,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="n">
         <v>135</v>
       </c>
@@ -3447,8 +3370,7 @@
       <c r="L56" t="n">
         <v>-100</v>
       </c>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="n">
+      <c r="M56" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -3478,7 +3400,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr"/>
       <c r="G57" t="n">
         <v>107</v>
       </c>
@@ -3501,8 +3422,7 @@
       <c r="L57" t="n">
         <v>-100</v>
       </c>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="n">
+      <c r="M57" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -3555,8 +3475,7 @@
       <c r="L58" t="n">
         <v>-100</v>
       </c>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="n">
+      <c r="M58" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -3609,8 +3528,7 @@
       <c r="L59" t="n">
         <v>90.91</v>
       </c>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="n">
+      <c r="M59" t="n">
         <v>45.45</v>
       </c>
     </row>
@@ -3663,8 +3581,7 @@
       <c r="L60" t="n">
         <v>0</v>
       </c>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="n">
+      <c r="M60" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3717,8 +3634,7 @@
       <c r="L61" t="n">
         <v>-100</v>
       </c>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="n">
+      <c r="M61" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -3771,8 +3687,7 @@
       <c r="L62" t="n">
         <v>95.23999999999999</v>
       </c>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="n">
+      <c r="M62" t="n">
         <v>47.62</v>
       </c>
     </row>
@@ -3819,10 +3734,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr"/>
-      <c r="L63" t="inlineStr"/>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3867,10 +3778,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr"/>
-      <c r="L64" t="inlineStr"/>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3921,8 +3828,7 @@
       <c r="L65" t="n">
         <v>120.5</v>
       </c>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="n">
+      <c r="M65" t="n">
         <v>60.25</v>
       </c>
     </row>
@@ -3975,8 +3881,7 @@
       <c r="L66" t="n">
         <v>54.05</v>
       </c>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="n">
+      <c r="M66" t="n">
         <v>27.03</v>
       </c>
     </row>
@@ -4029,8 +3934,7 @@
       <c r="L67" t="n">
         <v>106</v>
       </c>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="n">
+      <c r="M67" t="n">
         <v>53</v>
       </c>
     </row>
@@ -4083,8 +3987,7 @@
       <c r="L68" t="n">
         <v>-100</v>
       </c>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="n">
+      <c r="M68" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -4137,8 +4040,7 @@
       <c r="L69" t="n">
         <v>126.5</v>
       </c>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="n">
+      <c r="M69" t="n">
         <v>63.25</v>
       </c>
     </row>
@@ -4191,8 +4093,7 @@
       <c r="L70" t="n">
         <v>-100</v>
       </c>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="n">
+      <c r="M70" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -4245,8 +4146,7 @@
       <c r="L71" t="n">
         <v>60.79</v>
       </c>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="n">
+      <c r="M71" t="n">
         <v>30.4</v>
       </c>
     </row>
@@ -4299,8 +4199,7 @@
       <c r="L72" t="n">
         <v>54.95</v>
       </c>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="n">
+      <c r="M72" t="n">
         <v>27.47</v>
       </c>
     </row>
@@ -4353,8 +4252,7 @@
       <c r="L73" t="n">
         <v>-100</v>
       </c>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="n">
+      <c r="M73" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -4407,8 +4305,7 @@
       <c r="L74" t="n">
         <v>-100</v>
       </c>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="n">
+      <c r="M74" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -4461,8 +4358,7 @@
       <c r="L75" t="n">
         <v>125</v>
       </c>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="n">
+      <c r="M75" t="n">
         <v>62.5</v>
       </c>
     </row>
@@ -4515,8 +4411,7 @@
       <c r="L76" t="n">
         <v>80</v>
       </c>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="n">
+      <c r="M76" t="n">
         <v>40</v>
       </c>
     </row>
@@ -4569,8 +4464,7 @@
       <c r="L77" t="n">
         <v>-100</v>
       </c>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="n">
+      <c r="M77" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -4600,7 +4494,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="n">
         <v>102</v>
       </c>
@@ -4623,8 +4516,7 @@
       <c r="L78" t="n">
         <v>-100</v>
       </c>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="n">
+      <c r="M78" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -4654,7 +4546,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr"/>
       <c r="G79" t="n">
         <v>-129</v>
       </c>
@@ -4677,8 +4568,7 @@
       <c r="L79" t="n">
         <v>-100</v>
       </c>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="n">
+      <c r="M79" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -4708,7 +4598,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
       <c r="G80" t="n">
         <v>-155</v>
       </c>
@@ -4731,8 +4620,7 @@
       <c r="L80" t="n">
         <v>64.52</v>
       </c>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="n">
+      <c r="M80" t="n">
         <v>32.26</v>
       </c>
     </row>
@@ -4762,7 +4650,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr"/>
       <c r="G81" t="n">
         <v>118</v>
       </c>
@@ -4785,8 +4672,7 @@
       <c r="L81" t="n">
         <v>118</v>
       </c>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="n">
+      <c r="M81" t="n">
         <v>59</v>
       </c>
     </row>
@@ -4816,7 +4702,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr"/>
       <c r="G82" t="n">
         <v>-106</v>
       </c>
@@ -4839,8 +4724,7 @@
       <c r="L82" t="n">
         <v>94.34</v>
       </c>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="n">
+      <c r="M82" t="n">
         <v>47.17</v>
       </c>
     </row>
@@ -4870,7 +4754,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr"/>
       <c r="G83" t="n">
         <v>107.5</v>
       </c>
@@ -4893,8 +4776,7 @@
       <c r="L83" t="n">
         <v>107.5</v>
       </c>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="n">
+      <c r="M83" t="n">
         <v>53.75</v>
       </c>
     </row>
@@ -4947,8 +4829,7 @@
       <c r="L84" t="n">
         <v>90.91</v>
       </c>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="n">
+      <c r="M84" t="n">
         <v>45.45</v>
       </c>
     </row>
@@ -5001,8 +4882,7 @@
       <c r="L85" t="n">
         <v>95.23999999999999</v>
       </c>
-      <c r="M85" t="inlineStr"/>
-      <c r="N85" t="n">
+      <c r="M85" t="n">
         <v>47.62</v>
       </c>
     </row>
@@ -5055,8 +4935,7 @@
       <c r="L86" t="n">
         <v>-100</v>
       </c>
-      <c r="M86" t="inlineStr"/>
-      <c r="N86" t="n">
+      <c r="M86" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -5109,8 +4988,7 @@
       <c r="L87" t="n">
         <v>-100</v>
       </c>
-      <c r="M87" t="inlineStr"/>
-      <c r="N87" t="n">
+      <c r="M87" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -5163,8 +5041,7 @@
       <c r="L88" t="n">
         <v>-100</v>
       </c>
-      <c r="M88" t="inlineStr"/>
-      <c r="N88" t="n">
+      <c r="M88" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -5217,8 +5094,7 @@
       <c r="L89" t="n">
         <v>68.97</v>
       </c>
-      <c r="M89" t="inlineStr"/>
-      <c r="N89" t="n">
+      <c r="M89" t="n">
         <v>34.48</v>
       </c>
     </row>
@@ -5271,8 +5147,7 @@
       <c r="L90" t="n">
         <v>-100</v>
       </c>
-      <c r="M90" t="inlineStr"/>
-      <c r="N90" t="n">
+      <c r="M90" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -5325,8 +5200,7 @@
       <c r="L91" t="n">
         <v>54.5</v>
       </c>
-      <c r="M91" t="inlineStr"/>
-      <c r="N91" t="n">
+      <c r="M91" t="n">
         <v>27.25</v>
       </c>
     </row>
@@ -5356,7 +5230,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr"/>
       <c r="G92" t="n">
         <v>100</v>
       </c>
@@ -5379,8 +5252,7 @@
       <c r="L92" t="n">
         <v>-100</v>
       </c>
-      <c r="M92" t="inlineStr"/>
-      <c r="N92" t="n">
+      <c r="M92" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -5433,8 +5305,7 @@
       <c r="L93" t="n">
         <v>90.91</v>
       </c>
-      <c r="M93" t="inlineStr"/>
-      <c r="N93" t="n">
+      <c r="M93" t="n">
         <v>45.45</v>
       </c>
     </row>
@@ -5481,10 +5352,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr"/>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
-      <c r="N94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5535,8 +5402,7 @@
       <c r="L95" t="n">
         <v>-100</v>
       </c>
-      <c r="M95" t="inlineStr"/>
-      <c r="N95" t="n">
+      <c r="M95" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -5566,7 +5432,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="n">
         <v>-162</v>
       </c>
@@ -5589,8 +5454,7 @@
       <c r="L96" t="n">
         <v>-100</v>
       </c>
-      <c r="M96" t="inlineStr"/>
-      <c r="N96" t="n">
+      <c r="M96" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -5620,7 +5484,6 @@
           <t>AWAY</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
       <c r="G97" t="n">
         <v>217.5</v>
       </c>
@@ -5643,8 +5506,7 @@
       <c r="L97" t="n">
         <v>-100</v>
       </c>
-      <c r="M97" t="inlineStr"/>
-      <c r="N97" t="n">
+      <c r="M97" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -5697,8 +5559,7 @@
       <c r="L98" t="n">
         <v>82.3</v>
       </c>
-      <c r="M98" t="inlineStr"/>
-      <c r="N98" t="n">
+      <c r="M98" t="n">
         <v>41.15</v>
       </c>
     </row>
@@ -5751,8 +5612,7 @@
       <c r="L99" t="n">
         <v>-100</v>
       </c>
-      <c r="M99" t="inlineStr"/>
-      <c r="N99" t="n">
+      <c r="M99" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -5805,8 +5665,7 @@
       <c r="L100" t="n">
         <v>-100</v>
       </c>
-      <c r="M100" t="inlineStr"/>
-      <c r="N100" t="n">
+      <c r="M100" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -5853,10 +5712,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr"/>
-      <c r="L101" t="inlineStr"/>
-      <c r="M101" t="inlineStr"/>
-      <c r="N101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5907,8 +5762,7 @@
       <c r="L102" t="n">
         <v>-100</v>
       </c>
-      <c r="M102" t="inlineStr"/>
-      <c r="N102" t="n">
+      <c r="M102" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -5955,10 +5809,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr"/>
-      <c r="L103" t="inlineStr"/>
-      <c r="M103" t="inlineStr"/>
-      <c r="N103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6003,10 +5853,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr"/>
-      <c r="L104" t="inlineStr"/>
-      <c r="M104" t="inlineStr"/>
-      <c r="N104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -6057,8 +5903,7 @@
       <c r="L105" t="n">
         <v>92.59</v>
       </c>
-      <c r="M105" t="inlineStr"/>
-      <c r="N105" t="n">
+      <c r="M105" t="n">
         <v>46.3</v>
       </c>
     </row>
@@ -6105,12 +5950,10 @@
           <t>DNP</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr"/>
       <c r="L106" t="n">
         <v>0</v>
       </c>
-      <c r="M106" t="inlineStr"/>
-      <c r="N106" t="n">
+      <c r="M106" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6163,8 +6006,7 @@
       <c r="L107" t="n">
         <v>80.65000000000001</v>
       </c>
-      <c r="M107" t="inlineStr"/>
-      <c r="N107" t="n">
+      <c r="M107" t="n">
         <v>40.32</v>
       </c>
     </row>
@@ -6217,8 +6059,7 @@
       <c r="L108" t="n">
         <v>100</v>
       </c>
-      <c r="M108" t="inlineStr"/>
-      <c r="N108" t="n">
+      <c r="M108" t="n">
         <v>50</v>
       </c>
     </row>
@@ -6271,8 +6112,7 @@
       <c r="L109" t="n">
         <v>115</v>
       </c>
-      <c r="M109" t="inlineStr"/>
-      <c r="N109" t="n">
+      <c r="M109" t="n">
         <v>57.5</v>
       </c>
     </row>
@@ -6325,8 +6165,7 @@
       <c r="L110" t="n">
         <v>-100</v>
       </c>
-      <c r="M110" t="inlineStr"/>
-      <c r="N110" t="n">
+      <c r="M110" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -6379,8 +6218,7 @@
       <c r="L111" t="n">
         <v>84.75</v>
       </c>
-      <c r="M111" t="inlineStr"/>
-      <c r="N111" t="n">
+      <c r="M111" t="n">
         <v>42.37</v>
       </c>
     </row>
@@ -6433,8 +6271,7 @@
       <c r="L112" t="n">
         <v>72.45999999999999</v>
       </c>
-      <c r="M112" t="inlineStr"/>
-      <c r="N112" t="n">
+      <c r="M112" t="n">
         <v>36.23</v>
       </c>
     </row>
@@ -6481,10 +6318,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr"/>
-      <c r="L113" t="inlineStr"/>
-      <c r="M113" t="inlineStr"/>
-      <c r="N113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6535,8 +6368,7 @@
       <c r="L114" t="n">
         <v>109.5</v>
       </c>
-      <c r="M114" t="inlineStr"/>
-      <c r="N114" t="n">
+      <c r="M114" t="n">
         <v>54.75</v>
       </c>
     </row>
@@ -6583,10 +6415,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K115" t="inlineStr"/>
-      <c r="L115" t="inlineStr"/>
-      <c r="M115" t="inlineStr"/>
-      <c r="N115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6614,7 +6442,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F116" t="inlineStr"/>
       <c r="G116" t="n">
         <v>-162</v>
       </c>
@@ -6637,8 +6464,7 @@
       <c r="L116" t="n">
         <v>-100</v>
       </c>
-      <c r="M116" t="inlineStr"/>
-      <c r="N116" t="n">
+      <c r="M116" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -6668,7 +6494,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F117" t="inlineStr"/>
       <c r="G117" t="n">
         <v>-119</v>
       </c>
@@ -6691,8 +6516,7 @@
       <c r="L117" t="n">
         <v>-100</v>
       </c>
-      <c r="M117" t="inlineStr"/>
-      <c r="N117" t="n">
+      <c r="M117" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -6722,7 +6546,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F118" t="inlineStr"/>
       <c r="G118" t="n">
         <v>-155</v>
       </c>
@@ -6745,8 +6568,7 @@
       <c r="L118" t="n">
         <v>-100</v>
       </c>
-      <c r="M118" t="inlineStr"/>
-      <c r="N118" t="n">
+      <c r="M118" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -6799,8 +6621,7 @@
       <c r="L119" t="n">
         <v>38.46</v>
       </c>
-      <c r="M119" t="inlineStr"/>
-      <c r="N119" t="n">
+      <c r="M119" t="n">
         <v>19.23</v>
       </c>
     </row>
@@ -6853,8 +6674,7 @@
       <c r="L120" t="n">
         <v>47.62</v>
       </c>
-      <c r="M120" t="inlineStr"/>
-      <c r="N120" t="n">
+      <c r="M120" t="n">
         <v>23.81</v>
       </c>
     </row>
@@ -6907,8 +6727,7 @@
       <c r="L121" t="n">
         <v>-100</v>
       </c>
-      <c r="M121" t="inlineStr"/>
-      <c r="N121" t="n">
+      <c r="M121" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -6938,7 +6757,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" t="n">
         <v>-105</v>
       </c>
@@ -6961,8 +6779,7 @@
       <c r="L122" t="n">
         <v>95.23999999999999</v>
       </c>
-      <c r="M122" t="inlineStr"/>
-      <c r="N122" t="n">
+      <c r="M122" t="n">
         <v>47.62</v>
       </c>
     </row>
@@ -6992,7 +6809,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr"/>
       <c r="G123" t="n">
         <v>112.5</v>
       </c>
@@ -7015,8 +6831,7 @@
       <c r="L123" t="n">
         <v>-100</v>
       </c>
-      <c r="M123" t="inlineStr"/>
-      <c r="N123" t="n">
+      <c r="M123" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -7046,7 +6861,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F124" t="inlineStr"/>
       <c r="G124" t="n">
         <v>-195</v>
       </c>
@@ -7069,8 +6883,7 @@
       <c r="L124" t="n">
         <v>51.28</v>
       </c>
-      <c r="M124" t="inlineStr"/>
-      <c r="N124" t="n">
+      <c r="M124" t="n">
         <v>25.64</v>
       </c>
     </row>
@@ -7123,8 +6936,7 @@
       <c r="L125" t="n">
         <v>-100</v>
       </c>
-      <c r="M125" t="inlineStr"/>
-      <c r="N125" t="n">
+      <c r="M125" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -7177,8 +6989,7 @@
       <c r="L126" t="n">
         <v>-100</v>
       </c>
-      <c r="M126" t="inlineStr"/>
-      <c r="N126" t="n">
+      <c r="M126" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -7231,8 +7042,7 @@
       <c r="L127" t="n">
         <v>-100</v>
       </c>
-      <c r="M127" t="inlineStr"/>
-      <c r="N127" t="n">
+      <c r="M127" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -7285,8 +7095,7 @@
       <c r="L128" t="n">
         <v>-100</v>
       </c>
-      <c r="M128" t="inlineStr"/>
-      <c r="N128" t="n">
+      <c r="M128" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -7339,8 +7148,7 @@
       <c r="L129" t="n">
         <v>-100</v>
       </c>
-      <c r="M129" t="inlineStr"/>
-      <c r="N129" t="n">
+      <c r="M129" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -7393,8 +7201,7 @@
       <c r="L130" t="n">
         <v>62.11</v>
       </c>
-      <c r="M130" t="inlineStr"/>
-      <c r="N130" t="n">
+      <c r="M130" t="n">
         <v>31.06</v>
       </c>
     </row>
@@ -7447,8 +7254,7 @@
       <c r="L131" t="n">
         <v>-100</v>
       </c>
-      <c r="M131" t="inlineStr"/>
-      <c r="N131" t="n">
+      <c r="M131" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -7501,8 +7307,7 @@
       <c r="L132" t="n">
         <v>-100</v>
       </c>
-      <c r="M132" t="inlineStr"/>
-      <c r="N132" t="n">
+      <c r="M132" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -7555,8 +7360,7 @@
       <c r="L133" t="n">
         <v>52.63</v>
       </c>
-      <c r="M133" t="inlineStr"/>
-      <c r="N133" t="n">
+      <c r="M133" t="n">
         <v>26.32</v>
       </c>
     </row>
@@ -7603,12 +7407,10 @@
           <t>DNP</t>
         </is>
       </c>
-      <c r="K134" t="inlineStr"/>
       <c r="L134" t="n">
         <v>0</v>
       </c>
-      <c r="M134" t="inlineStr"/>
-      <c r="N134" t="n">
+      <c r="M134" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7661,8 +7463,7 @@
       <c r="L135" t="n">
         <v>68.97</v>
       </c>
-      <c r="M135" t="inlineStr"/>
-      <c r="N135" t="n">
+      <c r="M135" t="n">
         <v>34.48</v>
       </c>
     </row>
@@ -7715,8 +7516,7 @@
       <c r="L136" t="n">
         <v>-100</v>
       </c>
-      <c r="M136" t="inlineStr"/>
-      <c r="N136" t="n">
+      <c r="M136" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -7769,8 +7569,7 @@
       <c r="L137" t="n">
         <v>110.5</v>
       </c>
-      <c r="M137" t="inlineStr"/>
-      <c r="N137" t="n">
+      <c r="M137" t="n">
         <v>55.25</v>
       </c>
     </row>
@@ -7823,8 +7622,7 @@
       <c r="L138" t="n">
         <v>-100</v>
       </c>
-      <c r="M138" t="inlineStr"/>
-      <c r="N138" t="n">
+      <c r="M138" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -7877,8 +7675,7 @@
       <c r="L139" t="n">
         <v>-100</v>
       </c>
-      <c r="M139" t="inlineStr"/>
-      <c r="N139" t="n">
+      <c r="M139" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -7931,8 +7728,7 @@
       <c r="L140" t="n">
         <v>46.19</v>
       </c>
-      <c r="M140" t="inlineStr"/>
-      <c r="N140" t="n">
+      <c r="M140" t="n">
         <v>23.09</v>
       </c>
     </row>
@@ -7985,8 +7781,7 @@
       <c r="L141" t="n">
         <v>-100</v>
       </c>
-      <c r="M141" t="inlineStr"/>
-      <c r="N141" t="n">
+      <c r="M141" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -8039,8 +7834,7 @@
       <c r="L142" t="n">
         <v>63.69</v>
       </c>
-      <c r="M142" t="inlineStr"/>
-      <c r="N142" t="n">
+      <c r="M142" t="n">
         <v>31.85</v>
       </c>
     </row>
@@ -8093,8 +7887,7 @@
       <c r="L143" t="n">
         <v>-100</v>
       </c>
-      <c r="M143" t="inlineStr"/>
-      <c r="N143" t="n">
+      <c r="M143" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -8147,8 +7940,7 @@
       <c r="L144" t="n">
         <v>49.38</v>
       </c>
-      <c r="M144" t="inlineStr"/>
-      <c r="N144" t="n">
+      <c r="M144" t="n">
         <v>24.69</v>
       </c>
     </row>
@@ -8201,8 +7993,7 @@
       <c r="L145" t="n">
         <v>100.5</v>
       </c>
-      <c r="M145" t="inlineStr"/>
-      <c r="N145" t="n">
+      <c r="M145" t="n">
         <v>50.25</v>
       </c>
     </row>
@@ -8255,8 +8046,7 @@
       <c r="L146" t="n">
         <v>83.33</v>
       </c>
-      <c r="M146" t="inlineStr"/>
-      <c r="N146" t="n">
+      <c r="M146" t="n">
         <v>41.67</v>
       </c>
     </row>
@@ -8309,8 +8099,7 @@
       <c r="L147" t="n">
         <v>-100</v>
       </c>
-      <c r="M147" t="inlineStr"/>
-      <c r="N147" t="n">
+      <c r="M147" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -8363,8 +8152,7 @@
       <c r="L148" t="n">
         <v>-100</v>
       </c>
-      <c r="M148" t="inlineStr"/>
-      <c r="N148" t="n">
+      <c r="M148" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -8394,7 +8182,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F149" t="inlineStr"/>
       <c r="G149" t="n">
         <v>-102</v>
       </c>
@@ -8417,8 +8204,7 @@
       <c r="L149" t="n">
         <v>-100</v>
       </c>
-      <c r="M149" t="inlineStr"/>
-      <c r="N149" t="n">
+      <c r="M149" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -8448,7 +8234,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F150" t="inlineStr"/>
       <c r="G150" t="n">
         <v>110</v>
       </c>
@@ -8471,8 +8256,7 @@
       <c r="L150" t="n">
         <v>110</v>
       </c>
-      <c r="M150" t="inlineStr"/>
-      <c r="N150" t="n">
+      <c r="M150" t="n">
         <v>55</v>
       </c>
     </row>
@@ -8502,7 +8286,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr"/>
       <c r="G151" t="n">
         <v>-128</v>
       </c>
@@ -8525,8 +8308,7 @@
       <c r="L151" t="n">
         <v>78.12</v>
       </c>
-      <c r="M151" t="inlineStr"/>
-      <c r="N151" t="n">
+      <c r="M151" t="n">
         <v>39.06</v>
       </c>
     </row>
@@ -8556,7 +8338,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F152" t="inlineStr"/>
       <c r="G152" t="n">
         <v>-109</v>
       </c>
@@ -8579,8 +8360,7 @@
       <c r="L152" t="n">
         <v>91.73999999999999</v>
       </c>
-      <c r="M152" t="inlineStr"/>
-      <c r="N152" t="n">
+      <c r="M152" t="n">
         <v>45.87</v>
       </c>
     </row>
@@ -8610,7 +8390,6 @@
           <t>AWAY</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr"/>
       <c r="G153" t="n">
         <v>144.5</v>
       </c>
@@ -8633,8 +8412,7 @@
       <c r="L153" t="n">
         <v>144.5</v>
       </c>
-      <c r="M153" t="inlineStr"/>
-      <c r="N153" t="n">
+      <c r="M153" t="n">
         <v>72.25</v>
       </c>
     </row>
@@ -8687,8 +8465,7 @@
       <c r="L154" t="n">
         <v>-100</v>
       </c>
-      <c r="M154" t="inlineStr"/>
-      <c r="N154" t="n">
+      <c r="M154" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -8741,8 +8518,7 @@
       <c r="L155" t="n">
         <v>-100</v>
       </c>
-      <c r="M155" t="inlineStr"/>
-      <c r="N155" t="n">
+      <c r="M155" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -8795,8 +8571,7 @@
       <c r="L156" t="n">
         <v>80</v>
       </c>
-      <c r="M156" t="inlineStr"/>
-      <c r="N156" t="n">
+      <c r="M156" t="n">
         <v>40</v>
       </c>
     </row>
@@ -8849,8 +8624,7 @@
       <c r="L157" t="n">
         <v>-100</v>
       </c>
-      <c r="M157" t="inlineStr"/>
-      <c r="N157" t="n">
+      <c r="M157" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -8903,8 +8677,7 @@
       <c r="L158" t="n">
         <v>100</v>
       </c>
-      <c r="M158" t="inlineStr"/>
-      <c r="N158" t="n">
+      <c r="M158" t="n">
         <v>50</v>
       </c>
     </row>
@@ -8957,8 +8730,7 @@
       <c r="L159" t="n">
         <v>31.25</v>
       </c>
-      <c r="M159" t="inlineStr"/>
-      <c r="N159" t="n">
+      <c r="M159" t="n">
         <v>15.62</v>
       </c>
     </row>
@@ -9011,8 +8783,7 @@
       <c r="L160" t="n">
         <v>-100</v>
       </c>
-      <c r="M160" t="inlineStr"/>
-      <c r="N160" t="n">
+      <c r="M160" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -9065,8 +8836,7 @@
       <c r="L161" t="n">
         <v>57.14</v>
       </c>
-      <c r="M161" t="inlineStr"/>
-      <c r="N161" t="n">
+      <c r="M161" t="n">
         <v>28.57</v>
       </c>
     </row>
@@ -9119,8 +8889,7 @@
       <c r="L162" t="n">
         <v>71.43000000000001</v>
       </c>
-      <c r="M162" t="inlineStr"/>
-      <c r="N162" t="n">
+      <c r="M162" t="n">
         <v>35.71</v>
       </c>
     </row>
@@ -9173,8 +8942,7 @@
       <c r="L163" t="n">
         <v>58.82</v>
       </c>
-      <c r="M163" t="inlineStr"/>
-      <c r="N163" t="n">
+      <c r="M163" t="n">
         <v>29.41</v>
       </c>
     </row>
@@ -9227,8 +8995,7 @@
       <c r="L164" t="n">
         <v>-100</v>
       </c>
-      <c r="M164" t="inlineStr"/>
-      <c r="N164" t="n">
+      <c r="M164" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -9281,8 +9048,7 @@
       <c r="L165" t="n">
         <v>-100</v>
       </c>
-      <c r="M165" t="inlineStr"/>
-      <c r="N165" t="n">
+      <c r="M165" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -9335,8 +9101,7 @@
       <c r="L166" t="n">
         <v>-100</v>
       </c>
-      <c r="M166" t="inlineStr"/>
-      <c r="N166" t="n">
+      <c r="M166" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -9389,8 +9154,7 @@
       <c r="L167" t="n">
         <v>-100</v>
       </c>
-      <c r="M167" t="inlineStr"/>
-      <c r="N167" t="n">
+      <c r="M167" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -9443,8 +9207,7 @@
       <c r="L168" t="n">
         <v>82.3</v>
       </c>
-      <c r="M168" t="inlineStr"/>
-      <c r="N168" t="n">
+      <c r="M168" t="n">
         <v>41.15</v>
       </c>
     </row>
@@ -9497,8 +9260,7 @@
       <c r="L169" t="n">
         <v>50.89</v>
       </c>
-      <c r="M169" t="inlineStr"/>
-      <c r="N169" t="n">
+      <c r="M169" t="n">
         <v>25.45</v>
       </c>
     </row>
@@ -9528,7 +9290,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr"/>
       <c r="G170" t="n">
         <v>-100</v>
       </c>
@@ -9551,8 +9312,7 @@
       <c r="L170" t="n">
         <v>100</v>
       </c>
-      <c r="M170" t="inlineStr"/>
-      <c r="N170" t="n">
+      <c r="M170" t="n">
         <v>50</v>
       </c>
     </row>
@@ -9582,7 +9342,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F171" t="inlineStr"/>
       <c r="G171" t="n">
         <v>-102</v>
       </c>
@@ -9605,8 +9364,7 @@
       <c r="L171" t="n">
         <v>-100</v>
       </c>
-      <c r="M171" t="inlineStr"/>
-      <c r="N171" t="n">
+      <c r="M171" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -10224,12 +9982,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>pnl_50</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>pnl_50</t>
+          <t>git_commits</t>
         </is>
       </c>
     </row>
@@ -10259,7 +10017,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>100</v>
       </c>
@@ -10282,8 +10039,7 @@
       <c r="L2" t="n">
         <v>-100</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
+      <c r="M2" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -10313,7 +10069,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>-141.5</v>
       </c>
@@ -10336,8 +10091,7 @@
       <c r="L3" t="n">
         <v>70.67</v>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="n">
+      <c r="M3" t="n">
         <v>35.34</v>
       </c>
     </row>
@@ -10367,7 +10121,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
         <v>-121</v>
       </c>
@@ -10390,8 +10143,7 @@
       <c r="L4" t="n">
         <v>82.64</v>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
+      <c r="M4" t="n">
         <v>41.32</v>
       </c>
     </row>
@@ -10421,7 +10173,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>-156.5</v>
       </c>
@@ -10444,8 +10195,7 @@
       <c r="L5" t="n">
         <v>63.9</v>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="n">
+      <c r="M5" t="n">
         <v>31.95</v>
       </c>
     </row>
@@ -10475,7 +10225,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>135</v>
       </c>
@@ -10498,8 +10247,7 @@
       <c r="L6" t="n">
         <v>-100</v>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="n">
+      <c r="M6" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -10529,7 +10277,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>107</v>
       </c>
@@ -10552,8 +10299,7 @@
       <c r="L7" t="n">
         <v>-100</v>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
+      <c r="M7" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -10583,7 +10329,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
         <v>107.5</v>
       </c>
@@ -10606,8 +10351,7 @@
       <c r="L8" t="n">
         <v>107.5</v>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="n">
+      <c r="M8" t="n">
         <v>53.75</v>
       </c>
     </row>
@@ -10637,7 +10381,6 @@
           <t>AWAY</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>217.5</v>
       </c>
@@ -10660,8 +10403,7 @@
       <c r="L9" t="n">
         <v>-100</v>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="n">
+      <c r="M9" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -10691,7 +10433,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
         <v>112.5</v>
       </c>
@@ -10714,8 +10455,7 @@
       <c r="L10" t="n">
         <v>-100</v>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="n">
+      <c r="M10" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -10745,7 +10485,6 @@
           <t>HOME</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>-195</v>
       </c>
@@ -10768,8 +10507,7 @@
       <c r="L11" t="n">
         <v>51.28</v>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="n">
+      <c r="M11" t="n">
         <v>25.64</v>
       </c>
     </row>
@@ -10799,7 +10537,6 @@
           <t>AWAY</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>144.5</v>
       </c>
@@ -10822,8 +10559,7 @@
       <c r="L12" t="n">
         <v>144.5</v>
       </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="n">
+      <c r="M12" t="n">
         <v>72.25</v>
       </c>
     </row>
@@ -10904,12 +10640,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>pnl_50</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>pnl_50</t>
+          <t>git_commits</t>
         </is>
       </c>
     </row>
@@ -10962,8 +10698,7 @@
       <c r="L2" t="n">
         <v>-100</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
+      <c r="M2" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -11016,8 +10751,7 @@
       <c r="L3" t="n">
         <v>-100</v>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="n">
+      <c r="M3" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -11070,8 +10804,7 @@
       <c r="L4" t="n">
         <v>82.3</v>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
+      <c r="M4" t="n">
         <v>41.15</v>
       </c>
     </row>
@@ -11124,8 +10857,7 @@
       <c r="L5" t="n">
         <v>90.91</v>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="n">
+      <c r="M5" t="n">
         <v>45.45</v>
       </c>
     </row>
@@ -11178,8 +10910,7 @@
       <c r="L6" t="n">
         <v>95.23999999999999</v>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="n">
+      <c r="M6" t="n">
         <v>47.62</v>
       </c>
     </row>
@@ -11232,8 +10963,7 @@
       <c r="L7" t="n">
         <v>90.91</v>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
+      <c r="M7" t="n">
         <v>45.45</v>
       </c>
     </row>
@@ -11286,8 +11016,7 @@
       <c r="L8" t="n">
         <v>-100</v>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="n">
+      <c r="M8" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -11340,8 +11069,7 @@
       <c r="L9" t="n">
         <v>95.23999999999999</v>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="n">
+      <c r="M9" t="n">
         <v>47.62</v>
       </c>
     </row>
@@ -11394,8 +11122,7 @@
       <c r="L10" t="n">
         <v>90.91</v>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="n">
+      <c r="M10" t="n">
         <v>45.45</v>
       </c>
     </row>
@@ -11448,8 +11175,7 @@
       <c r="L11" t="n">
         <v>-100</v>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="n">
+      <c r="M11" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -11502,8 +11228,7 @@
       <c r="L12" t="n">
         <v>86.95999999999999</v>
       </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="n">
+      <c r="M12" t="n">
         <v>43.48</v>
       </c>
     </row>
@@ -11556,8 +11281,7 @@
       <c r="L13" t="n">
         <v>94.34</v>
       </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="n">
+      <c r="M13" t="n">
         <v>47.17</v>
       </c>
     </row>
@@ -11610,8 +11334,7 @@
       <c r="L14" t="n">
         <v>82.64</v>
       </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="n">
+      <c r="M14" t="n">
         <v>41.32</v>
       </c>
     </row>
@@ -11664,8 +11387,7 @@
       <c r="L15" t="n">
         <v>95.23999999999999</v>
       </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="n">
+      <c r="M15" t="n">
         <v>47.62</v>
       </c>
     </row>
@@ -11718,8 +11440,7 @@
       <c r="L16" t="n">
         <v>0</v>
       </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
+      <c r="M16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -11772,8 +11493,7 @@
       <c r="L17" t="n">
         <v>-100</v>
       </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="n">
+      <c r="M17" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -11826,8 +11546,7 @@
       <c r="L18" t="n">
         <v>-100</v>
       </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="n">
+      <c r="M18" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -11880,8 +11599,7 @@
       <c r="L19" t="n">
         <v>-100</v>
       </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="n">
+      <c r="M19" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -11934,8 +11652,7 @@
       <c r="L20" t="n">
         <v>-100</v>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="n">
+      <c r="M20" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -11988,8 +11705,7 @@
       <c r="L21" t="n">
         <v>-100</v>
       </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
+      <c r="M21" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -12070,12 +11786,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>pnl_50</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>pnl_50</t>
+          <t>git_commits</t>
         </is>
       </c>
     </row>
@@ -12128,8 +11844,7 @@
       <c r="L2" t="n">
         <v>62.7</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
+      <c r="M2" t="n">
         <v>31.35</v>
       </c>
     </row>
@@ -12182,8 +11897,7 @@
       <c r="L3" t="n">
         <v>95.23999999999999</v>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="n">
+      <c r="M3" t="n">
         <v>47.62</v>
       </c>
     </row>
@@ -12236,8 +11950,7 @@
       <c r="L4" t="n">
         <v>-100</v>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
+      <c r="M4" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -12290,8 +12003,7 @@
       <c r="L5" t="n">
         <v>60.61</v>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="n">
+      <c r="M5" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -12344,8 +12056,7 @@
       <c r="L6" t="n">
         <v>86.95999999999999</v>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="n">
+      <c r="M6" t="n">
         <v>43.48</v>
       </c>
     </row>
@@ -12398,8 +12109,7 @@
       <c r="L7" t="n">
         <v>-100</v>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
+      <c r="M7" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -12446,10 +12156,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12500,8 +12206,7 @@
       <c r="L9" t="n">
         <v>62.11</v>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="n">
+      <c r="M9" t="n">
         <v>31.06</v>
       </c>
     </row>
@@ -12554,8 +12259,7 @@
       <c r="L10" t="n">
         <v>-100</v>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="n">
+      <c r="M10" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -12602,10 +12306,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12656,8 +12356,7 @@
       <c r="L12" t="n">
         <v>-100</v>
       </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="n">
+      <c r="M12" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -12710,8 +12409,7 @@
       <c r="L13" t="n">
         <v>-100</v>
       </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="n">
+      <c r="M13" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -12764,8 +12462,7 @@
       <c r="L14" t="n">
         <v>60.79</v>
       </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="n">
+      <c r="M14" t="n">
         <v>30.4</v>
       </c>
     </row>
@@ -12818,8 +12515,7 @@
       <c r="L15" t="n">
         <v>-100</v>
       </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="n">
+      <c r="M15" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -12872,8 +12568,7 @@
       <c r="L16" t="n">
         <v>54.95</v>
       </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
+      <c r="M16" t="n">
         <v>27.47</v>
       </c>
     </row>
@@ -12920,10 +12615,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -12974,8 +12665,7 @@
       <c r="L18" t="n">
         <v>-100</v>
       </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="n">
+      <c r="M18" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -13028,8 +12718,7 @@
       <c r="L19" t="n">
         <v>-100</v>
       </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="n">
+      <c r="M19" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -13082,8 +12771,7 @@
       <c r="L20" t="n">
         <v>-100</v>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="n">
+      <c r="M20" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -13130,12 +12818,10 @@
           <t>DNP</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
         <v>0</v>
       </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
+      <c r="M21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13182,10 +12868,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13236,8 +12918,7 @@
       <c r="L23" t="n">
         <v>92.59</v>
       </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="n">
+      <c r="M23" t="n">
         <v>46.3</v>
       </c>
     </row>
@@ -13290,8 +12971,7 @@
       <c r="L24" t="n">
         <v>126.5</v>
       </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="n">
+      <c r="M24" t="n">
         <v>63.25</v>
       </c>
     </row>
@@ -13344,8 +13024,7 @@
       <c r="L25" t="n">
         <v>80.65000000000001</v>
       </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="n">
+      <c r="M25" t="n">
         <v>40.32</v>
       </c>
     </row>
@@ -13398,8 +13077,7 @@
       <c r="L26" t="n">
         <v>100</v>
       </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="n">
+      <c r="M26" t="n">
         <v>50</v>
       </c>
     </row>
@@ -13452,8 +13130,7 @@
       <c r="L27" t="n">
         <v>115</v>
       </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="n">
+      <c r="M27" t="n">
         <v>57.5</v>
       </c>
     </row>
@@ -13506,8 +13183,7 @@
       <c r="L28" t="n">
         <v>-100</v>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="n">
+      <c r="M28" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -13560,8 +13236,7 @@
       <c r="L29" t="n">
         <v>84.75</v>
       </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="n">
+      <c r="M29" t="n">
         <v>42.37</v>
       </c>
     </row>
@@ -13614,8 +13289,7 @@
       <c r="L30" t="n">
         <v>72.45999999999999</v>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="n">
+      <c r="M30" t="n">
         <v>36.23</v>
       </c>
     </row>
@@ -13668,8 +13342,7 @@
       <c r="L31" t="n">
         <v>38.46</v>
       </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="n">
+      <c r="M31" t="n">
         <v>19.23</v>
       </c>
     </row>
@@ -13722,8 +13395,7 @@
       <c r="L32" t="n">
         <v>47.62</v>
       </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="n">
+      <c r="M32" t="n">
         <v>23.81</v>
       </c>
     </row>
@@ -13770,10 +13442,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
-      <c r="L33" t="inlineStr"/>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -13824,8 +13492,7 @@
       <c r="L34" t="n">
         <v>-100</v>
       </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="n">
+      <c r="M34" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -13878,8 +13545,7 @@
       <c r="L35" t="n">
         <v>68.97</v>
       </c>
-      <c r="M35" t="inlineStr"/>
-      <c r="N35" t="n">
+      <c r="M35" t="n">
         <v>34.48</v>
       </c>
     </row>
@@ -13932,8 +13598,7 @@
       <c r="L36" t="n">
         <v>54.05</v>
       </c>
-      <c r="M36" t="inlineStr"/>
-      <c r="N36" t="n">
+      <c r="M36" t="n">
         <v>27.03</v>
       </c>
     </row>
@@ -13986,8 +13651,7 @@
       <c r="L37" t="n">
         <v>106</v>
       </c>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="n">
+      <c r="M37" t="n">
         <v>53</v>
       </c>
     </row>
@@ -14040,8 +13704,7 @@
       <c r="L38" t="n">
         <v>-100</v>
       </c>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="n">
+      <c r="M38" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -14094,8 +13757,7 @@
       <c r="L39" t="n">
         <v>-100</v>
       </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="n">
+      <c r="M39" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -14148,8 +13810,7 @@
       <c r="L40" t="n">
         <v>70.92</v>
       </c>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="n">
+      <c r="M40" t="n">
         <v>35.46</v>
       </c>
     </row>
@@ -14202,8 +13863,7 @@
       <c r="L41" t="n">
         <v>-100</v>
       </c>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="n">
+      <c r="M41" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -14256,8 +13916,7 @@
       <c r="L42" t="n">
         <v>-100</v>
       </c>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="n">
+      <c r="M42" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -14310,8 +13969,7 @@
       <c r="L43" t="n">
         <v>65.15000000000001</v>
       </c>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="n">
+      <c r="M43" t="n">
         <v>32.57</v>
       </c>
     </row>
@@ -14364,8 +14022,7 @@
       <c r="L44" t="n">
         <v>-100</v>
       </c>
-      <c r="M44" t="inlineStr"/>
-      <c r="N44" t="n">
+      <c r="M44" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -14418,8 +14075,7 @@
       <c r="L45" t="n">
         <v>66.67</v>
       </c>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="n">
+      <c r="M45" t="n">
         <v>33.33</v>
       </c>
     </row>
@@ -14472,8 +14128,7 @@
       <c r="L46" t="n">
         <v>57.14</v>
       </c>
-      <c r="M46" t="inlineStr"/>
-      <c r="N46" t="n">
+      <c r="M46" t="n">
         <v>28.57</v>
       </c>
     </row>
@@ -14526,8 +14181,7 @@
       <c r="L47" t="n">
         <v>73.8</v>
       </c>
-      <c r="M47" t="inlineStr"/>
-      <c r="N47" t="n">
+      <c r="M47" t="n">
         <v>36.9</v>
       </c>
     </row>
@@ -14580,8 +14234,7 @@
       <c r="L48" t="n">
         <v>-100</v>
       </c>
-      <c r="M48" t="inlineStr"/>
-      <c r="N48" t="n">
+      <c r="M48" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -14628,10 +14281,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="inlineStr"/>
-      <c r="M49" t="inlineStr"/>
-      <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -14682,8 +14331,7 @@
       <c r="L50" t="n">
         <v>-100</v>
       </c>
-      <c r="M50" t="inlineStr"/>
-      <c r="N50" t="n">
+      <c r="M50" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -14736,8 +14384,7 @@
       <c r="L51" t="n">
         <v>-100</v>
       </c>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="n">
+      <c r="M51" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -14784,10 +14431,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr"/>
-      <c r="M52" t="inlineStr"/>
-      <c r="N52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -14832,10 +14475,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
-      <c r="L53" t="inlineStr"/>
-      <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -14886,8 +14525,7 @@
       <c r="L54" t="n">
         <v>58.82</v>
       </c>
-      <c r="M54" t="inlineStr"/>
-      <c r="N54" t="n">
+      <c r="M54" t="n">
         <v>29.41</v>
       </c>
     </row>
@@ -14940,8 +14578,7 @@
       <c r="L55" t="n">
         <v>-100</v>
       </c>
-      <c r="M55" t="inlineStr"/>
-      <c r="N55" t="n">
+      <c r="M55" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -14994,8 +14631,7 @@
       <c r="L56" t="n">
         <v>120.5</v>
       </c>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="n">
+      <c r="M56" t="n">
         <v>60.25</v>
       </c>
     </row>
@@ -15048,8 +14684,7 @@
       <c r="L57" t="n">
         <v>54.05</v>
       </c>
-      <c r="M57" t="inlineStr"/>
-      <c r="N57" t="n">
+      <c r="M57" t="n">
         <v>27.03</v>
       </c>
     </row>
@@ -15102,8 +14737,7 @@
       <c r="L58" t="n">
         <v>-100</v>
       </c>
-      <c r="M58" t="inlineStr"/>
-      <c r="N58" t="n">
+      <c r="M58" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -15156,8 +14790,7 @@
       <c r="L59" t="n">
         <v>-100</v>
       </c>
-      <c r="M59" t="inlineStr"/>
-      <c r="N59" t="n">
+      <c r="M59" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -15210,8 +14843,7 @@
       <c r="L60" t="n">
         <v>80</v>
       </c>
-      <c r="M60" t="inlineStr"/>
-      <c r="N60" t="n">
+      <c r="M60" t="n">
         <v>40</v>
       </c>
     </row>
@@ -15264,8 +14896,7 @@
       <c r="L61" t="n">
         <v>57.14</v>
       </c>
-      <c r="M61" t="inlineStr"/>
-      <c r="N61" t="n">
+      <c r="M61" t="n">
         <v>28.57</v>
       </c>
     </row>
@@ -15318,8 +14949,7 @@
       <c r="L62" t="n">
         <v>-100</v>
       </c>
-      <c r="M62" t="inlineStr"/>
-      <c r="N62" t="n">
+      <c r="M62" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -15372,8 +15002,7 @@
       <c r="L63" t="n">
         <v>-100</v>
       </c>
-      <c r="M63" t="inlineStr"/>
-      <c r="N63" t="n">
+      <c r="M63" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -15426,8 +15055,7 @@
       <c r="L64" t="n">
         <v>31.25</v>
       </c>
-      <c r="M64" t="inlineStr"/>
-      <c r="N64" t="n">
+      <c r="M64" t="n">
         <v>15.62</v>
       </c>
     </row>
@@ -15480,8 +15108,7 @@
       <c r="L65" t="n">
         <v>100</v>
       </c>
-      <c r="M65" t="inlineStr"/>
-      <c r="N65" t="n">
+      <c r="M65" t="n">
         <v>50</v>
       </c>
     </row>
@@ -15534,8 +15161,7 @@
       <c r="L66" t="n">
         <v>-100</v>
       </c>
-      <c r="M66" t="inlineStr"/>
-      <c r="N66" t="n">
+      <c r="M66" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -15588,8 +15214,7 @@
       <c r="L67" t="n">
         <v>80</v>
       </c>
-      <c r="M67" t="inlineStr"/>
-      <c r="N67" t="n">
+      <c r="M67" t="n">
         <v>40</v>
       </c>
     </row>
@@ -15642,8 +15267,7 @@
       <c r="L68" t="n">
         <v>-100</v>
       </c>
-      <c r="M68" t="inlineStr"/>
-      <c r="N68" t="n">
+      <c r="M68" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -15696,8 +15320,7 @@
       <c r="L69" t="n">
         <v>-100</v>
       </c>
-      <c r="M69" t="inlineStr"/>
-      <c r="N69" t="n">
+      <c r="M69" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -15750,8 +15373,7 @@
       <c r="L70" t="n">
         <v>63.69</v>
       </c>
-      <c r="M70" t="inlineStr"/>
-      <c r="N70" t="n">
+      <c r="M70" t="n">
         <v>31.85</v>
       </c>
     </row>
@@ -15804,8 +15426,7 @@
       <c r="L71" t="n">
         <v>46.19</v>
       </c>
-      <c r="M71" t="inlineStr"/>
-      <c r="N71" t="n">
+      <c r="M71" t="n">
         <v>23.09</v>
       </c>
     </row>
@@ -15858,8 +15479,7 @@
       <c r="L72" t="n">
         <v>68.97</v>
       </c>
-      <c r="M72" t="inlineStr"/>
-      <c r="N72" t="n">
+      <c r="M72" t="n">
         <v>34.48</v>
       </c>
     </row>
@@ -15912,8 +15532,7 @@
       <c r="L73" t="n">
         <v>-100</v>
       </c>
-      <c r="M73" t="inlineStr"/>
-      <c r="N73" t="n">
+      <c r="M73" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -15966,8 +15585,7 @@
       <c r="L74" t="n">
         <v>110.5</v>
       </c>
-      <c r="M74" t="inlineStr"/>
-      <c r="N74" t="n">
+      <c r="M74" t="n">
         <v>55.25</v>
       </c>
     </row>
@@ -16020,8 +15638,7 @@
       <c r="L75" t="n">
         <v>-100</v>
       </c>
-      <c r="M75" t="inlineStr"/>
-      <c r="N75" t="n">
+      <c r="M75" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -16068,12 +15685,10 @@
           <t>DNP</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr"/>
       <c r="L76" t="n">
         <v>0</v>
       </c>
-      <c r="M76" t="inlineStr"/>
-      <c r="N76" t="n">
+      <c r="M76" t="n">
         <v>0</v>
       </c>
     </row>
@@ -16126,8 +15741,7 @@
       <c r="L77" t="n">
         <v>52.63</v>
       </c>
-      <c r="M77" t="inlineStr"/>
-      <c r="N77" t="n">
+      <c r="M77" t="n">
         <v>26.32</v>
       </c>
     </row>
@@ -16180,8 +15794,7 @@
       <c r="L78" t="n">
         <v>-100</v>
       </c>
-      <c r="M78" t="inlineStr"/>
-      <c r="N78" t="n">
+      <c r="M78" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -16234,8 +15847,7 @@
       <c r="L79" t="n">
         <v>-100</v>
       </c>
-      <c r="M79" t="inlineStr"/>
-      <c r="N79" t="n">
+      <c r="M79" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -16288,8 +15900,7 @@
       <c r="L80" t="n">
         <v>62.11</v>
       </c>
-      <c r="M80" t="inlineStr"/>
-      <c r="N80" t="n">
+      <c r="M80" t="n">
         <v>31.06</v>
       </c>
     </row>
@@ -16342,8 +15953,7 @@
       <c r="L81" t="n">
         <v>-100</v>
       </c>
-      <c r="M81" t="inlineStr"/>
-      <c r="N81" t="n">
+      <c r="M81" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -16396,8 +16006,7 @@
       <c r="L82" t="n">
         <v>71.43000000000001</v>
       </c>
-      <c r="M82" t="inlineStr"/>
-      <c r="N82" t="n">
+      <c r="M82" t="n">
         <v>35.71</v>
       </c>
     </row>
@@ -16450,8 +16059,7 @@
       <c r="L83" t="n">
         <v>-100</v>
       </c>
-      <c r="M83" t="inlineStr"/>
-      <c r="N83" t="n">
+      <c r="M83" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -16504,8 +16112,7 @@
       <c r="L84" t="n">
         <v>58.82</v>
       </c>
-      <c r="M84" t="inlineStr"/>
-      <c r="N84" t="n">
+      <c r="M84" t="n">
         <v>29.41</v>
       </c>
     </row>
@@ -16586,12 +16193,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>pnl_50</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>pnl_50</t>
+          <t>git_commits</t>
         </is>
       </c>
     </row>
@@ -16644,8 +16251,7 @@
       <c r="L2" t="n">
         <v>100</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
+      <c r="M2" t="n">
         <v>50</v>
       </c>
     </row>
@@ -16692,10 +16298,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -16746,8 +16348,7 @@
       <c r="L4" t="n">
         <v>-100</v>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
+      <c r="M4" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -16794,10 +16395,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -16848,8 +16445,7 @@
       <c r="L6" t="n">
         <v>109.5</v>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="n">
+      <c r="M6" t="n">
         <v>54.75</v>
       </c>
     </row>
@@ -16896,10 +16492,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -16950,8 +16542,7 @@
       <c r="L8" t="n">
         <v>-100</v>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="n">
+      <c r="M8" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -17004,8 +16595,7 @@
       <c r="L9" t="n">
         <v>-100</v>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="n">
+      <c r="M9" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -17058,8 +16648,7 @@
       <c r="L10" t="n">
         <v>80</v>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="n">
+      <c r="M10" t="n">
         <v>40</v>
       </c>
     </row>
@@ -17112,8 +16701,7 @@
       <c r="L11" t="n">
         <v>125</v>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="n">
+      <c r="M11" t="n">
         <v>62.5</v>
       </c>
     </row>
@@ -17166,8 +16754,7 @@
       <c r="L12" t="n">
         <v>-100</v>
       </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="n">
+      <c r="M12" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -17220,8 +16807,7 @@
       <c r="L13" t="n">
         <v>54.5</v>
       </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="n">
+      <c r="M13" t="n">
         <v>27.25</v>
       </c>
     </row>
@@ -17274,8 +16860,7 @@
       <c r="L14" t="n">
         <v>-100</v>
       </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="n">
+      <c r="M14" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -17328,8 +16913,7 @@
       <c r="L15" t="n">
         <v>-100</v>
       </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="n">
+      <c r="M15" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -17382,8 +16966,7 @@
       <c r="L16" t="n">
         <v>59.7</v>
       </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
+      <c r="M16" t="n">
         <v>29.85</v>
       </c>
     </row>
@@ -17430,10 +17013,6 @@
           <t>ODDS_ERR</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -17484,8 +17063,7 @@
       <c r="L18" t="n">
         <v>-100</v>
       </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="n">
+      <c r="M18" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -17538,8 +17116,7 @@
       <c r="L19" t="n">
         <v>90.91</v>
       </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="n">
+      <c r="M19" t="n">
         <v>45.45</v>
       </c>
     </row>
@@ -17592,8 +17169,7 @@
       <c r="L20" t="n">
         <v>-100</v>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="n">
+      <c r="M20" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -17646,8 +17222,7 @@
       <c r="L21" t="n">
         <v>145</v>
       </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
+      <c r="M21" t="n">
         <v>72.5</v>
       </c>
     </row>
@@ -17700,8 +17275,7 @@
       <c r="L22" t="n">
         <v>57.14</v>
       </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="n">
+      <c r="M22" t="n">
         <v>28.57</v>
       </c>
     </row>
@@ -17754,8 +17328,7 @@
       <c r="L23" t="n">
         <v>-100</v>
       </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="n">
+      <c r="M23" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -17808,8 +17381,7 @@
       <c r="L24" t="n">
         <v>-100</v>
       </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="n">
+      <c r="M24" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -17862,8 +17434,7 @@
       <c r="L25" t="n">
         <v>-100</v>
       </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="n">
+      <c r="M25" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -17916,8 +17487,7 @@
       <c r="L26" t="n">
         <v>-100</v>
       </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="n">
+      <c r="M26" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -17970,8 +17540,7 @@
       <c r="L27" t="n">
         <v>-100</v>
       </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="n">
+      <c r="M27" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -18024,8 +17593,7 @@
       <c r="L28" t="n">
         <v>49.38</v>
       </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="n">
+      <c r="M28" t="n">
         <v>24.69</v>
       </c>
     </row>
@@ -18078,8 +17646,7 @@
       <c r="L29" t="n">
         <v>-100</v>
       </c>
-      <c r="M29" t="inlineStr"/>
-      <c r="N29" t="n">
+      <c r="M29" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -18132,8 +17699,7 @@
       <c r="L30" t="n">
         <v>83.33</v>
       </c>
-      <c r="M30" t="inlineStr"/>
-      <c r="N30" t="n">
+      <c r="M30" t="n">
         <v>41.67</v>
       </c>
     </row>
@@ -18186,8 +17752,7 @@
       <c r="L31" t="n">
         <v>100.5</v>
       </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="n">
+      <c r="M31" t="n">
         <v>50.25</v>
       </c>
     </row>
@@ -18240,8 +17805,7 @@
       <c r="L32" t="n">
         <v>82.3</v>
       </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="n">
+      <c r="M32" t="n">
         <v>41.15</v>
       </c>
     </row>
@@ -18294,8 +17858,7 @@
       <c r="L33" t="n">
         <v>-100</v>
       </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="n">
+      <c r="M33" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -18348,8 +17911,7 @@
       <c r="L34" t="n">
         <v>50.89</v>
       </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="n">
+      <c r="M34" t="n">
         <v>25.45</v>
       </c>
     </row>
@@ -18430,12 +17992,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>pnl_50</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>pnl_50</t>
+          <t>git_commits</t>
         </is>
       </c>
     </row>
@@ -18465,7 +18027,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>-157.5</v>
       </c>
@@ -18488,8 +18049,7 @@
       <c r="L2" t="n">
         <v>63.49</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="n">
+      <c r="M2" t="n">
         <v>31.75</v>
       </c>
     </row>
@@ -18519,7 +18079,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
         <v>120</v>
       </c>
@@ -18542,8 +18101,7 @@
       <c r="L3" t="n">
         <v>-100</v>
       </c>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="n">
+      <c r="M3" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -18573,7 +18131,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
         <v>-105</v>
       </c>
@@ -18596,8 +18153,7 @@
       <c r="L4" t="n">
         <v>95.23999999999999</v>
       </c>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
+      <c r="M4" t="n">
         <v>47.62</v>
       </c>
     </row>
@@ -18627,7 +18183,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
         <v>-155</v>
       </c>
@@ -18650,8 +18205,7 @@
       <c r="L5" t="n">
         <v>-100</v>
       </c>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="n">
+      <c r="M5" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -18681,7 +18235,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>-119</v>
       </c>
@@ -18704,8 +18257,7 @@
       <c r="L6" t="n">
         <v>-100</v>
       </c>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="n">
+      <c r="M6" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -18735,7 +18287,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
         <v>-162</v>
       </c>
@@ -18758,8 +18309,7 @@
       <c r="L7" t="n">
         <v>-100</v>
       </c>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="n">
+      <c r="M7" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -18789,7 +18339,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
         <v>-162</v>
       </c>
@@ -18812,8 +18361,7 @@
       <c r="L8" t="n">
         <v>-100</v>
       </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="n">
+      <c r="M8" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -18843,7 +18391,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>-106</v>
       </c>
@@ -18866,8 +18413,7 @@
       <c r="L9" t="n">
         <v>94.34</v>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="n">
+      <c r="M9" t="n">
         <v>47.17</v>
       </c>
     </row>
@@ -18897,7 +18443,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
         <v>118</v>
       </c>
@@ -18920,8 +18465,7 @@
       <c r="L10" t="n">
         <v>118</v>
       </c>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="n">
+      <c r="M10" t="n">
         <v>59</v>
       </c>
     </row>
@@ -18951,7 +18495,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>100</v>
       </c>
@@ -18974,8 +18517,7 @@
       <c r="L11" t="n">
         <v>-100</v>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="n">
+      <c r="M11" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -19005,7 +18547,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>-129</v>
       </c>
@@ -19028,8 +18569,7 @@
       <c r="L12" t="n">
         <v>-100</v>
       </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="n">
+      <c r="M12" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -19059,7 +18599,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
         <v>102</v>
       </c>
@@ -19082,8 +18621,7 @@
       <c r="L13" t="n">
         <v>-100</v>
       </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="n">
+      <c r="M13" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -19113,7 +18651,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
         <v>106</v>
       </c>
@@ -19136,8 +18673,7 @@
       <c r="L14" t="n">
         <v>-100</v>
       </c>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="n">
+      <c r="M14" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -19167,7 +18703,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
         <v>-112</v>
       </c>
@@ -19190,8 +18725,7 @@
       <c r="L15" t="n">
         <v>-100</v>
       </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="n">
+      <c r="M15" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -19221,7 +18755,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="n">
         <v>-102</v>
       </c>
@@ -19244,8 +18777,7 @@
       <c r="L16" t="n">
         <v>98.04000000000001</v>
       </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
+      <c r="M16" t="n">
         <v>49.02</v>
       </c>
     </row>
@@ -19275,7 +18807,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="n">
         <v>120</v>
       </c>
@@ -19298,8 +18829,7 @@
       <c r="L17" t="n">
         <v>120</v>
       </c>
-      <c r="M17" t="inlineStr"/>
-      <c r="N17" t="n">
+      <c r="M17" t="n">
         <v>60</v>
       </c>
     </row>
@@ -19329,7 +18859,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="n">
         <v>-155</v>
       </c>
@@ -19352,8 +18881,7 @@
       <c r="L18" t="n">
         <v>64.52</v>
       </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="n">
+      <c r="M18" t="n">
         <v>32.26</v>
       </c>
     </row>
@@ -19383,7 +18911,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="n">
         <v>-100</v>
       </c>
@@ -19406,8 +18933,7 @@
       <c r="L19" t="n">
         <v>100</v>
       </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="n">
+      <c r="M19" t="n">
         <v>50</v>
       </c>
     </row>
@@ -19437,7 +18963,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="n">
         <v>-102</v>
       </c>
@@ -19460,8 +18985,7 @@
       <c r="L20" t="n">
         <v>-100</v>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="n">
+      <c r="M20" t="n">
         <v>-50</v>
       </c>
     </row>
@@ -19491,7 +19015,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
         <v>110</v>
       </c>
@@ -19514,8 +19037,7 @@
       <c r="L21" t="n">
         <v>110</v>
       </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
+      <c r="M21" t="n">
         <v>55</v>
       </c>
     </row>
@@ -19545,7 +19067,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
         <v>-128</v>
       </c>
@@ -19568,8 +19089,7 @@
       <c r="L22" t="n">
         <v>78.12</v>
       </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="n">
+      <c r="M22" t="n">
         <v>39.06</v>
       </c>
     </row>
@@ -19599,7 +19119,6 @@
           <t>NRFI</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="n">
         <v>-109</v>
       </c>
@@ -19622,8 +19141,7 @@
       <c r="L23" t="n">
         <v>91.73999999999999</v>
       </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="n">
+      <c r="M23" t="n">
         <v>45.87</v>
       </c>
     </row>
@@ -19653,7 +19171,6 @@
           <t>YRFI</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="n">
         <v>-102</v>
       </c>
@@ -19676,8 +19193,7 @@
       <c r="L24" t="n">
         <v>-100</v>
       </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="n">
+      <c r="M24" t="n">
         <v>-50</v>
       </c>
     </row>

</xml_diff>